<commit_message>
fix(deploy): sync index.html and render_dashboard.html, add /sw.js route, and purge service worker stale cache
</commit_message>
<xml_diff>
--- a/reports/Daily_Report_2026-09-03.xlsx
+++ b/reports/Daily_Report_2026-09-03.xlsx
@@ -553,7 +553,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated on 2026-09-03 22:50:27 IST</t>
+          <t>Generated on 2026-09-03 23:04:23 IST</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>0.15%</t>
+          <t>0.40%</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="B22" s="14" t="n">
-        <v>0.5435814049320037</v>
+        <v>0.5425700124478694</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">

</xml_diff>